<commit_message>
Update version compatibility files
</commit_message>
<xml_diff>
--- a/version_compatibility/Compatibility Summary.xlsx
+++ b/version_compatibility/Compatibility Summary.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dponti/GitHub/validation/version_compatibility/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{D36C7AA7-DE05-1844-9A83-09D25CEAE952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67E60674-8177-334C-91C7-2C297A80688F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5160" yWindow="8120" windowWidth="49840" windowHeight="19800" xr2:uid="{304F4BEB-B345-284F-90E5-3B53C3058EF7}"/>
+    <workbookView xWindow="5240" yWindow="4260" windowWidth="49840" windowHeight="25940" xr2:uid="{304F4BEB-B345-284F-90E5-3B53C3058EF7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="149">
   <si>
     <t>Issue</t>
   </si>
@@ -322,9 +321,6 @@
 ComponentLithology/@association</t>
   </si>
   <si>
-    <t>The diggs:Lithology object is no longer used for describe the characteristics of a lithology component. A new diggs:ComponentLith object is used in its stead. Enumerated values for @association have changed to simpler phrases.</t>
-  </si>
-  <si>
     <t>Component Lithology restructuring</t>
   </si>
   <si>
@@ -358,12 +354,555 @@
     &lt;/constituent&gt;
 &lt;/ConstituentObservation&gt;</t>
   </si>
+  <si>
+    <t>Dictionary Restrictions</t>
+  </si>
+  <si>
+    <t>diggs:Definition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is used only in DIGGS dictionariesl any properly designed custom dictionaries will have the gml:name and gml:descriptionpopulate and will not be using deprecated elements. This change does not effect+E13+E13 DIGGS xml instances. </t>
+  </si>
+  <si>
+    <t>&lt;diggs:Definition gml:id="submitted"&gt;
+    &lt;gml:description&gt;Testing schedule has been submitted&lt;/gml:description&gt;
+    &lt;gml:identifier codeSpace="https://diggsml.org/def/authorities.xml#DIGGS"&gt;https://diggsml.org/def/codes/DIGGS/0.1/progressState.xml#submitted&lt;/gml:identifier&gt;
+    &lt;gml:name&gt;Submitted&lt;/gml:name&gt;
+    &lt;diggs:dataType&gt;string&lt;/diggs:dataType&gt;
+    &lt;diggs:occurrences&gt;
+        &lt;diggs:Occurrence&gt;
+            &lt;diggs:sourceElementXpath&gt;//diggs:testingProgress//diggs:state&lt;/diggs:sourceElementXpath&gt;
+        &lt;/diggs:Occurrence&gt;
+        &lt;diggs:Occurrence&gt; &lt;diggs:sourceElementXpath&gt;//diggs:scheduleProgress//diggs:state&lt;/diggs:sourceElementXpath&gt;
+        &lt;/diggs:Occurrence&gt;
+    &lt;/diggs:occurrences&gt;
+&lt;/diggs:Definition&gt;</t>
+  </si>
+  <si>
+    <t>&lt;diggs:Definition gml:id="submitted"&gt;
+    &lt;gml:identifier codeSpace="https://diggsml.org/def/authorities.xml#DIGGS"&gt;https://diggsml.org/def/codes/DIGGS/0.1/progressState.xml#submitted&lt;/gml:identifier&gt;
+    &lt;diggs:dataType&gt;string&lt;/diggs:dataType&gt;
+    &lt;diggs:occurrences&gt;
+        &lt;diggs:Occurrence&gt;
+            &lt;diggs:sourceElementXpath&gt;//diggs:testingProgress//diggs:state&lt;/diggs:sourceElementXpath&gt;
+        &lt;/diggs:Occurrence&gt;
+        &lt;diggs:Occurrence&gt; &lt;
+             diggs:sourceElementXpath&gt;//diggs:scheduleProgress//diggs:state&lt;/diggs:sourceElementXpath&gt;
+        &lt;/diggs:Occurrence&gt;
+    &lt;/diggs:occurrences&gt;
+&lt;/diggs:Definition&gt;</t>
+  </si>
+  <si>
+    <t>DelayEvent Restriction</t>
+  </si>
+  <si>
+    <t>diggs:DelayEvent</t>
+  </si>
+  <si>
+    <t>diggs:timeOfDelay or diggs:delayDuration now required.</t>
+  </si>
+  <si>
+    <t>Make sure timeOfDelay or delayDuration are present in object. Well formed DelayEvent in 2.6 should already have timeOfDelay</t>
+  </si>
+  <si>
+    <t>&lt;diggs:DelayEvent gml:id="de1"&gt;
+  &lt;diggs:timeOfDelay&gt;
+    &lt;diggs:TimeInterval gml:id="fi1"&gt;
+      &lt;diggs:start&gt;02:10:45&lt;/diggs:start&gt;
+      &lt;diggs:end&gt;02:11:00&lt;/diggs:end&gt;
+  &lt;/diggs:TimeInterval&gt;
+&lt;/diggs:timeOfDelay&gt;
+&lt;/diggs:DelayEvent&gt;</t>
+  </si>
+  <si>
+    <t>&lt;diggs:DelayEvent gml:id="de1"&gt;
+ &lt;/diggs:DelayEvent&gt;</t>
+  </si>
+  <si>
+    <t>legendCode attribute removal</t>
+  </si>
+  <si>
+    <t>diggs:Color/diggs:colorCode
+diggs:Color/diggs:colorName
+diggs:Constituent/diggs:codeVlaue
+diggs:Lithology:classificationCode</t>
+  </si>
+  <si>
+    <t>Properties gml:name and gml:description now mandatory. gml:descriptionReference (deprecated in gml 3.2.1) )is removed.</t>
+  </si>
+  <si>
+    <t>Attribute legendCode in type DescriptorCodeType, deprecated in 2.6, is now removed.</t>
+  </si>
+  <si>
+    <t>The attribute is not relevant to Color or Constituent - remove. For Lithology, use legendCode property for the value instead.</t>
+  </si>
+  <si>
+    <t>&lt;diggs:Lithology gml:id="l1"&gt;
+  &lt;diggs:classificationCode codeSpace="http://diggsml.org/def/codes/DIGGS/0.1/astmD2487.xml#GC" legendCode="GC"&gt;Clayey gravel&lt;/diggs:classificationCode&gt;
+&lt;/diggs:Lithology&gt;</t>
+  </si>
+  <si>
+    <t>&lt;diggs:Lithology gml:id="l1"&gt;
+  &lt;diggs:classificationCode codeSpace="http://diggsml.org/def/codes/DIGGS/0.1/astmD2487.xml#GC"&gt;Clayey gravel&lt;/diggs:classificationCode&gt;
+  &lt;diggs:legendCode&gt;GC&lt;/diggs:legendCode
+&lt;/diggs:Lithology&gt;</t>
+  </si>
+  <si>
+    <t>Property Renaming</t>
+  </si>
+  <si>
+    <t>diggs:DesignGroutMix</t>
+  </si>
+  <si>
+    <t>Property diggs:pressureFiltrationValueDesign renamed to diggs:pressureFiltrationCoefficientDesign</t>
+  </si>
+  <si>
+    <t>&lt;diggs:pressureFiltrationCoefficientDesign&gt;0.4&lt;/diggspressureFiltrationCoefficientDesign&gt;</t>
+  </si>
+  <si>
+    <t>&lt;diggs:pressureFiltrationValueDesign&gt;0.4&lt;/diggspressureFiltrationValueDesign</t>
+  </si>
+  <si>
+    <t>Change property to new name.</t>
+  </si>
+  <si>
+    <t>Qualified attribue @diggs:howDetermined changed to unqualified howDetermined</t>
+  </si>
+  <si>
+    <t>Change @diggs:howDetermined to @howDetermined</t>
+  </si>
+  <si>
+    <t>&lt;diggs:LithologyObservation diggs:howDetermined="visual" gml:id="lo1" &gt;
+    …
+&lt;diggs:LithologyObservation&gt;</t>
+  </si>
+  <si>
+    <t>&lt;diggs:LithologyObservation howDetermined="visual" gml:id="lo1" &gt;
+    …
+&lt;diggs:LithologyObservation&gt;</t>
+  </si>
+  <si>
+    <t>diggs:ColorObservation
+diggs:ConstituentObservation
+diggs:DiscontinuityObservation
+diggs:GeoUnitObservation
+diggs:LithologyObservation
+diggsOrientationObservation
+diggs:OtherObservation
+diggs:StratigraphyObservation</t>
+  </si>
+  <si>
+    <t>Attribute qualification change</t>
+  </si>
+  <si>
+    <t>Envrionment Restrictions</t>
+  </si>
+  <si>
+    <t>diggs:Environment</t>
+  </si>
+  <si>
+    <t>Removed diggs: gasFlow and diggs: gasPressure properties from Environment object</t>
+  </si>
+  <si>
+    <t>Remove these properties from instance</t>
+  </si>
+  <si>
+    <t>&lt;diggs:Environment gml:id="env1"&gt;
+  &lt;diggs:gasFlow uom="l/min"&gt;0.2&lt;/diggs:gasFlow&gt;
+  &lt;diggs:humidity uom="%"&gt;54.2&lt;/diggs:humidity&gt;
+  &lt;diggs:gasPressure uom="psi"&gt;18&lt;/diggs:gasPressure&gt;
+  &lt;diggs:weather&gt;sunny&lt;/diggs:weather&gt;
+ &lt;/diggs:Environment&gt;</t>
+  </si>
+  <si>
+    <t>&lt;diggs:Environment gml:id="env1"&gt;
+  &lt;diggs:humidity uom="%"&gt;54.2&lt;/diggs:humidity&gt;
+   &lt;diggs:weather&gt;sunny&lt;/diggs:weather&gt;
+ &lt;/diggs:Environment&gt;</t>
+  </si>
+  <si>
+    <t>FieldProperties changes</t>
+  </si>
+  <si>
+    <t>Change names of renamed elements and remove those properties that were removed. Restrict cardinality of particle properties to a single replication of each (highly unlikely in existing instances)</t>
+  </si>
+  <si>
+    <t>diggs:Lithology/diggs:fieldProperties
+diggs:FieldProperties</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> diggs:lithologydiggs:/fieldProperties name changed to diggs:Lithologydiggs:/lithProperties; diggs:FieldProperties name changed to diggs:LithProperties; diggs:otherFIeldProperty name changed to diggs:otherLithProperty; diggs:particleSizeMaximum removed (incorportated into new property); gml:status and gml:name removed. Cardinality restricted for diggs:particleAngularity, diggs:particleHardness, diggs;particleShape, diggs:particleSize.</t>
+  </si>
+  <si>
+    <t>&lt;diggs:fieldProperties&gt;
+  &lt;diggs:FieldProperties gml:id="fp1"&gt;
+    &lt;diggs:particleAngularity codeSpace="ASTM" sizeClass="sand"&gt;subrounded&lt;/diggs:particleAngularity&gt;
+    &lt;diggs:particleAngularity codeSpace="ASTM" sizeClass="gravel"&gt;angular&lt;/diggs:particleAngularity&gt;
+    &lt;diggs:particleHardness codeSpace="ASTM" sizeClass="sand"&gt;hard&lt;/diggs:particleHardness&gt;
+    &lt;diggs:particleShape codeSpace="ASTM" sizeClass="sand"&gt;spherical&lt;/diggs:particleShape&gt;
+    &lt;diggs:particleSize codeSpace="ASTM" sizeClass="sand"&gt;fine to medium&lt;/diggs:particleSize&gt;
+    &lt;diggs:particleSizeMaximum&gt;4 mm&lt;/diggs:particleSizeMaximum&gt;
+    &lt;diggs:otherFieldProperty&gt;
+        &lt;diggs:Parameter&gt;
+            &lt;diggs:parameterName&gt;taste&lt;/diggs:parameterName&gt;
+                &lt;diggs:parameterValue&gt;salty&lt;/diggs:parameterValue&gt;
+        &lt;/diggs:Parameter&gt;
+    &lt;/diggs:otherFieldProperty&gt;
+  &lt;/diggs:FieldProperties&gt;
+&lt;/diggs:fieldProperties&gt;</t>
+  </si>
+  <si>
+    <t>&lt;diggs:lithProperties&gt;
+    &lt;diggs:LithProperties gml:id="fp1"&gt;
+        &lt;diggs:particleAngularity codeSpace="ASTM"&gt;subrounded to angular&lt;/diggs:particleAngularity&gt;
+        &lt;diggs:particleHardness codeSpace="ASTM"&gt;hard&lt;/diggs:particleHardness&gt;
+        &lt;diggs:particleShape codeSpace="ASTM"&gt;spherical&lt;/diggs:particleShape&gt;
+        &lt;diggs:particleSize codeSpace="ASTM"&gt;fine to medium&lt;/diggs:particleSize&gt;
+        &lt;diggs:particleSizeDistribution&gt;
+            &lt;diggs:ParticleSizeDistribution&gt;
+                &lt;maximumDiameter&gt;
+                    &lt;ParticleSize gml:id="ps1"&gt;
+                      &lt;particleSizeValue uom="mm"&gt;4&lt;/particleSizeValue&gt;
+                    &lt;/ParticleSize&gt;
+                &lt;/maximumDiameter&gt;
+            &lt;/diggs:ParticleSizeDistribution&gt;
+        &lt;/diggs:particleSizeDistribution&gt;
+        &lt;diggs:otherLithProperty&gt;
+            &lt;diggs:Parameter&gt;
+                &lt;diggs:parameterName&gt;taste&lt;/diggs:parameterName&gt;
+                &lt;diggs:parameterValue&gt;salty&lt;/diggs:parameterValue&gt;
+            &lt;/diggs:Parameter&gt;
+        &lt;/diggs:otherLithProperty&gt;
+    &lt;/diggs:LithProperties&gt;
+&lt;/diggs:lithProperties&gt;</t>
+  </si>
+  <si>
+    <t>Frost Susceptibility Test restructuring</t>
+  </si>
+  <si>
+    <t>diggs:FrostSusceptibilityTest</t>
+  </si>
+  <si>
+    <t>Test restructured to include  diggs:FrostHeaveTrial objects instead of fixed diggs:frostHaave1, diggs:FrostHeave2, etc.properties. Specimen metadata moved to specimen object. Restructuring allows for multiple specimen metadata associeated with each heave value.</t>
+  </si>
+  <si>
+    <t>Create SoilSpecimenObjects for each specimen tested - add metadata there, and place frostHeave1, frostHeave2 into separate trial objects.</t>
+  </si>
+  <si>
+    <t>&lt;FrostSusceptibilityTest gml:id="FrostSusceptibilityTest_dlc_ld1_k3c"&gt;
+    &lt;specimen&gt;
+        &lt;SoilSpecimen gml:id="pk3_k21"&gt;
+            &lt;sampleRef xlink:href="#samp1"/&gt;
+             &lt;conditionPreTest&gt;
+                 &lt;SpecimenConditions gml:id="sc1"&gt;
+                     &lt;dryUnitWeight uom="g/cm3"&gt;2.1&lt;/dryUnitWeight&gt;
+                     &lt;waterContent uom="%"&gt;35&lt;/waterContent&gt;
+                 &lt;/SpecimenConditions&gt;
+             &lt;/conditionPreTest&gt;
+        &lt;/SoilSpecimen&gt;
+    &lt;/specimen&gt;
+    &lt;specimen&gt;
+        &lt;SoilSpecimen gml:id="g1r_w21"&gt;
+            &lt;sampleRef xlink:href="#samp2"/&gt;
+            &lt;conditionPreTest&gt;
+                &lt;SpecimenConditions gml:id="sc2"&gt;
+                    &lt;dryUnitWeight uom="g/cm3"&gt;2.2&lt;/dryUnitWeight&gt;
+                    &lt;waterContent uom="%"&gt;23&lt;/waterContent&gt;
+                &lt;/SpecimenConditions&gt;
+            &lt;/conditionPreTest&gt;
+        &lt;/SoilSpecimen&gt;
+    &lt;/specimen&gt;
+    &lt;dryDensity uom="g/cm3"&gt;2.1&lt;/dryDensity&gt;
+    &lt;waterContent uom="%"&gt;25&lt;/waterContent&gt;
+    &lt;frostHeave1 uom="cm"&gt;1.2&lt;/frostHeave1&gt;
+    &lt;frostHeave2 uom="cm"&gt;0.97&lt;/frostHeave2&gt;
+&lt;/FrostSusceptibilityTest&gt;</t>
+  </si>
+  <si>
+    <t>&lt;FrostSusceptibilityTest gml:id="FrostSusceptibilityTest_dlc_ld1_k3c"&gt;
+    &lt;specimen&gt;
+        &lt;SoilSpecimen gml:id="pk3_k21"&gt;
+            &lt;sampleRef xlink:href="#samp1"/&gt;
+            &lt;conditionPreTest&gt;
+                &lt;SpecimenConditions gml:id="sc1"&gt;
+                    &lt;dryUnitWeight uom="g/cm3"&gt;2.1&lt;/dryUnitWeight&gt;
+                    &lt;waterContent uom="%"&gt;35&lt;/waterContent&gt;
+                &lt;/SpecimenConditions&gt;
+            &lt;/conditionPreTest&gt;
+        &lt;/SoilSpecimen&gt;
+    &lt;/specimen&gt;
+    &lt;specimen&gt;
+        &lt;SoilSpecimen gml:id="g1r_w21"&gt;
+            &lt;sampleRef xlink:href="#samp2"/&gt;
+            &lt;conditionPreTest&gt;
+                &lt;SpecimenConditions gml:id="sc2"&gt;
+                    &lt;dryUnitWeight uom="g/cm3"&gt;2.2&lt;/dryUnitWeight&gt;
+                    &lt;waterContent uom="%"&gt;23&lt;/waterContent&gt;
+                &lt;/SpecimenConditions&gt;
+            &lt;/conditionPreTest&gt;
+        &lt;/SoilSpecimen&gt;
+    &lt;/specimen&gt;
+    &lt;frostHeaveTrial&gt;
+        &lt;FrostHeaveTrial&gt;
+            &lt;specimenRef xlink:href="#pk3_k21"/&gt;
+            &lt;frostHeave uom="cm"&gt;1.2&lt;/frostHeave&gt;
+        &lt;/FrostHeaveTrial&gt;
+    &lt;/frostHeaveTrial&gt;
+    &lt;frostHeaveTrial&gt;
+        &lt;FrostHeaveTrial&gt;
+            &lt;specimenRef xlink:href="#g1r_w21"/&gt;
+            &lt;frostHeave uom="cm"&gt;0.97&lt;/frostHeave&gt;
+        &lt;/FrostHeaveTrial&gt;
+    &lt;/frostHeaveTrial&gt;
+&lt;/FrostSusceptibilityTest&gt;</t>
+  </si>
+  <si>
+    <t>Grout Grading Specification Changes</t>
+  </si>
+  <si>
+    <t>diggs:GroutGradingSpecification</t>
+  </si>
+  <si>
+    <t>The type for this element  now extends diggs:SieveAnalysisType instead of deprecated diggs_geo:SieveAnalysisType</t>
+  </si>
+  <si>
+    <t>Change namespace prefixes of all properties to diggs: namespace instead of diggs_geo,</t>
+  </si>
+  <si>
+    <t>&lt;diggs:GroutGradingSpecification gml:id="ggs1"&gt;
+  &lt;diggs_geo:coarseFractionWetSieved&gt;{0,1}true&lt;/diggs_geo:coarseFractionWetSieved&gt;
+  &lt;diggs_geo:gradingData&gt;
+  ...
+  &lt;/diggs_geo:gradingData&gt;
+  &lt;diggs_geo:panData&gt;
+  ...
+  &lt;/diggs_geo:panData&gt;
+&lt;/diggs:GroutGradingSpecification&gt;</t>
+  </si>
+  <si>
+    <t>&lt;diggs:GroutGradingSpecification gml:id="ggs1"&gt;
+  &lt;diggs:coarseFractionWetSieved&gt;{0,1}true&lt;/diggs_geo:coarseFractionWetSieved&gt;
+  &lt;diggs:gradingData&gt;
+  ...
+  &lt;/diggs:gradingData&gt;
+  &lt;diggs:panData&gt;
+  ...
+  &lt;/diggs:panData&gt;
+&lt;/diggs:GroutGradingSpecification&gt;</t>
+  </si>
+  <si>
+    <t>diggsGroutTrenchCutoffWall</t>
+  </si>
+  <si>
+    <t>Object modified to allow for linearly varying wall section depths</t>
+  </si>
+  <si>
+    <t>Replace unt yped depthIncrement property with wallSectionDepths array property type property.</t>
+  </si>
+  <si>
+    <t>&lt;diggs:GroutTrenchCutoffWall gml:id="cuw-1"&gt;
+  &lt;diggs:projectRef xlink:href="#proj1"/&gt;
+  &lt;diggs:referencePoint
+    &lt;diggs:PointLocation gml:id="pl-1"&gt;...&lt;/PointLocation
+  &lt;/diggs:referencePoint&gt;
+  &lt;diggs:centerLine&gt;
+    &lt;diggs:LinearExtent gml;i"le-1"&gt;...&lt;/diggs:LinearExtent&gt;
+  &lt;/diggs:centerLine&gt;
+  &lt;diggs:cutoffWallWidth uom="in"&gt;36&lt;/diggs:cutoffWallWidth&gt;
+  &lt;diggs:wallSectionDepths&gt;
+    &lt;diggs:CutoffWallSectionDepth gml:id="cuw-1-1"&gt;
+      &lt;diggs:sectionLocation&gt;
+        &lt;diggs:LinearExtent gml;i"le-2"&gt;...&lt;/diggs:LinearExtent&gt;
+      &lt;/diggs:sectionLocation&gt;
+      &lt;diggs:wallDepth uom="m"&gt;2&lt;/diggs:wallDepth&gt;
+    &lt;/diggs:CutoffWallSectionDepth&gt;
+    &lt;diggs:CutoffWallSectionDepth gml:id="cuw-1-2"&gt;
+      &lt;diggs:sectionLocation&gt;
+        &lt;diggs:LinearExtent gml;i"le-3"&gt;...&lt;/diggs:LinearExtent&gt;
+      &lt;/diggs:sectionLocation&gt;
+      &lt;diggs:wallDepth uom="m"&gt;2.5&lt;/diggs:wallDepth&gt;
+    &lt;/diggs:CutoffWallSectionDepth&gt;
+  &lt;/diggs:wallSectionDepths&gt;
+&lt;/diggs:GroutTrenchCutoffWall&gt;</t>
+  </si>
+  <si>
+    <t>&lt;diggs:GroutTrenchCutoffWall gml:id="cuw-1"&gt;
+  &lt;diggs:projectRef xlink:href="#proj1"/&gt;
+  &lt;diggs:referencePoint
+    &lt;diggs:PointLocation gml:id="pl-1"&gt;...&lt;/PointLocation
+  &lt;/diggs:referencePoint&gt;
+  &lt;diggs:centerLine&gt;
+    &lt;diggs:LinearExtent gml;i"le-1"&gt;...&lt;/diggs:LinearExtent&gt;
+  &lt;/diggs:centerLine&gt;
+  &lt;diggs:cutoffWallWidth uom="in"&gt;36&lt;/diggs:cutoffWallWidth&gt;
+  &lt;depthIncrement&gt;2&lt;depthIncrement
+&lt;/diggs:GroutTrenchCutoffWall&gt;</t>
+  </si>
+  <si>
+    <t>Grout Trench Cutoff Wall Changes</t>
+  </si>
+  <si>
+    <t>Limit Modifications</t>
+  </si>
+  <si>
+    <t>diggs:Limit</t>
+  </si>
+  <si>
+    <t>diggs:Limit now contains a mandatory outOfLimitValue property</t>
+  </si>
+  <si>
+    <t>Must add a representation of the value when it it out of imit.</t>
+  </si>
+  <si>
+    <t>&lt;diggs:Limit&gt;
+  &lt;diggs:limitType&gt;less than&lt;/diggs:limitType&gt;
+  &lt;diggs:value&gt;12&lt;diggs:value&gt;
+  &lt;diggs:outOfLimitValue&gt;&amp;lt;12&lt;/diggs:outOfLimitValue&gt;
+&lt;/diggs:Limit&gt;'</t>
+  </si>
+  <si>
+    <t>&lt;diggs:Limit&gt;
+  &lt;diggs:limitType&gt;less than&lt;/diggs:limitType&gt;
+  &lt;diggs:value&gt;12&lt;diggs:value&gt;
+&lt;/diggs:Limit&gt;</t>
+  </si>
+  <si>
+    <t>Lithology Modifications</t>
+  </si>
+  <si>
+    <t>diggs:Lithology</t>
+  </si>
+  <si>
+    <t>Improved structure of diggs:Lithology, including addition of componentLithology requires diggs:facies property moved to diggs:LithologyObservation, renaming of diggs:fieldProperties to diggs:lithProperties, renaming diggs:grainSizeDistribution to diggs:particleSizeDistribution and moving this property to diggs:LithProperties</t>
+  </si>
+  <si>
+    <t>The diggs:Lithology object is no longer used for describe the characteristics of a lithology component. A new diggs:ComponentLith object is used instead. Enumerated values for @association have changed to simpler phrases.</t>
+  </si>
+  <si>
+    <t>&lt;diggs:LithologyObservation gml:id="Litho_Soil_Observation_BH-33_0.5"&gt;
+	&lt;diggs:location&gt;
+		&lt;diggs:LinearExtent gml:id="DGS2A7E-4ED-FA5-2907-2A63" srsName="#lsr-BH-33"
+			srsDimension="1"&gt;
+			&lt;gml:posList&gt;3.0 11.0&lt;/gml:posList&gt;
+		&lt;/diggs:LinearExtent&gt;
+	&lt;/diggs:location&gt;
+	&lt;diggs:primaryLithology&gt;
+		&lt;diggs:Lithology gml:id="DGS14E4-D53-C4-71B0-3FB08"&gt;
+			&lt;diggs:classificationCode codeSpace="https://diggsml.org/def/codes/DIGGS/0.1/astmD2488.xml#GP-GCscb"&gt;Poorly graded gravel with clay and sand, Cobbles and Boulders&lt;/diggs:classificationCode&gt;
+			&lt;diggs:lithProperties&gt;
+				&lt;diggs:LithProperties gml:id="DGS3F43-164B-28A5-ABD7-41353"&gt;
+					&lt;diggs:consistency&gt;medium dense&lt;/diggs:consistency&gt;
+					&lt;diggs:cementation&gt;moderate&lt;/diggs:cementation&gt;
+					&lt;diggs:moistureCondition&gt;moist to wet&lt;/diggs:moistureCondition&gt;
+					&lt;diggs:odor&gt;no&lt;/diggs:odor&gt;
+					&lt;diggs:particleSorting&gt;poorly graded&lt;/diggs:particleSorting&gt;
+					&lt;diggs:reactionToHCl&gt;weak&lt;/diggs:reactionToHCl&gt;
+					&lt;diggs:soilStructure&gt;stratified&lt;/diggs:soilStructure&gt;
+				&lt;/diggs:LithProperties&gt;
+			&lt;/diggs:lithProperties&gt;
+		&lt;/diggs:Lithology&gt;
+	&lt;/diggs:primaryLithology&gt;
+	&lt;facies&gt;fill&lt;/facies&gt;
+&lt;/diggs:LithologyObservation&gt;</t>
+  </si>
+  <si>
+    <t>&lt;diggs:LithologyObservation gml:id="Litho_Soil_Observation_BH-33_0.5"&gt;
+    &lt;diggs:location&gt;
+        &lt;diggs:LinearExtent gml:id="DGS2A7E-4ED-FA5-2907-2A63" srsName="#lsr-BH-33"
+            srsDimension="1"&gt;
+            &lt;gml:posList&gt;3.0 11.0&lt;/gml:posList&gt;
+        &lt;/diggs:LinearExtent&gt;
+    &lt;/diggs:location&gt;
+    &lt;diggs:primaryLithology&gt;
+        &lt;diggs:Lithology gml:id="DGS14E4-D53-C4-71B0-3FB08"&gt;
+            &lt;diggs:classificationCode codeSpace="https://diggsml.org/def/codes/DIGGS/0.1/astmD2488.xml#GP-GCscb"&gt;Poorly graded gravel with clay and sand, Cobbles and Boulders&lt;/diggs:classificationCode&gt;
+            &lt;facies&gt;fill&lt;/facies&gt;
+            &lt;diggs:fieldProperties&gt;
+                &lt;diggs:FieldProperties gml:id="DGS3F43-164B-28A5-ABD7-41353"&gt;
+                    &lt;diggs:consistency&gt;medium dense&lt;/diggs:consistency&gt;
+                    &lt;diggs:cementation&gt;moderate&lt;/diggs:cementation&gt;
+                    &lt;diggs:moistureCondition&gt;moist to wet&lt;/diggs:moistureCondition&gt;
+                    &lt;diggs:odor&gt;no&lt;/diggs:odor&gt;
+                    &lt;diggs:particleSorting&gt;poorly graded&lt;/diggs:particleSorting&gt;
+                    &lt;diggs:reactionToHCl&gt;weak&lt;/diggs:reactionToHCl&gt;
+                    &lt;diggs:soilStructure&gt;stratified&lt;/diggs:soilStructure&gt;
+                &lt;/diggs:FieldProperties&gt;
+            &lt;/diggs:fieldProperties&gt;
+        &lt;/diggs:Lithology&gt;
+    &lt;/diggs:primaryLithology&gt;
+&lt;/diggs:LithologyObservation&gt;</t>
+  </si>
+  <si>
+    <t>Local Coordinate change</t>
+  </si>
+  <si>
+    <t>diggs:LocalCoordinate</t>
+  </si>
+  <si>
+    <t>Optional property originAxisAzimuth removed</t>
+  </si>
+  <si>
+    <t>This property doesn't fully describe rotated axes. In 3.0, use location property and define the local coordinate system in the diggs:crs property of diggs:DocumentInformation</t>
+  </si>
+  <si>
+    <t>&lt;diggs:LocalCoordinate&gt;
+  &lt;diggs:easting uom="m"&gt;10&lt;/diggs:easting&gt;
+  &lt;diggs:northing uom="m"&gt;8&lt;/diggs:northing&gt;
+  &lt;diggs:elevation uom="m"&gt;1.4&lt;/diggs:elevation&gt;
+  &lt;diggs:originAxisAzimuth refAzimuth="true north" uom="dega"&gt;10&lt;/diggs:originAxisAzimuth&gt;
+&lt;/diggs:LocalCoordinate&gt;</t>
+  </si>
+  <si>
+    <t>&lt;diggs:LocalCoordinate&gt;
+  &lt;diggs:location&gt;
+    &lt;diggs:PointLocation srsName="#localCRS" srsDimension="3"&gt; &lt;!-- Points to CRS defined in diggs:DocumentInformation/crs --&gt;
+      &lt;gml:pos&gt;10 8 1.4&lt;/gml:pos&gt;
+    &lt;/diggs:PointLocation&gt;
+  &lt;/diggs:location&gt;
+&lt;/diggs:LocalCoordinate&gt;</t>
+  </si>
+  <si>
+    <t>Location Uncertainty modifications</t>
+  </si>
+  <si>
+    <t>diggs:LocationUncertainty</t>
+  </si>
+  <si>
+    <t>Values of diggs:locationMethod property now comes from an enumerated list, instead of a possible coe list.</t>
+  </si>
+  <si>
+    <t>Map any currently used values for diggs:locationMethod to one of the enum values</t>
+  </si>
+  <si>
+    <t>&lt;diggs:LocationUncertainty gml:id="lu1"&gt;
+  &lt;diggs:locationMethod codeSpace="ODOT"&gt;gps&lt;/diggs:locationMethod&gt;
+  &lt;diggs:xValueUncertainty&gt;
+    &lt;diggs:Uncertainty gml:id="u1"&gt;
+      &lt;diggs:plusUncertaintyValue&gt;0.05&lt;/diggs:plusUncertaintyValue&gt;
+  &lt;diggs:minusUncertaintyValue&gt;0.05&lt;/diggs:minusUncertaintyValue&gt;
+  &lt;diggs:confidenceLevel uom="%"&gt;95&lt;/diggs:confidenceLevel&gt;
+&lt;/diggs:Uncertainty&gt;
+  &lt;/diggs:xValueUncertainty&gt;
+&lt;/diggs:LocationUncertainty&gt;</t>
+  </si>
+  <si>
+    <t>&lt;diggs:LocationUncertainty gml:id="lu1""&gt;
+  &lt;diggs:locationMethod"&gt;gnss&lt;/diggs:locationMethod&gt;
+  &lt;diggs:xValueUncertainty&gt;
+    &lt;diggs:Uncertainty gml:id="u1"&gt;
+      &lt;diggs:plusUncertaintyValue&gt;0.05&lt;/diggs:plusUncertaintyValue&gt;
+  &lt;diggs:minusUncertaintyValue&gt;0.05&lt;/diggs:minusUncertaintyValue&gt;
+  &lt;diggs:confidenceLevel uom="%"&gt;95&lt;/diggs:confidenceLevel&gt;
+&lt;/diggs:Uncertainty&gt;
+  &lt;/diggs:xValueUncertainty&gt;
+&lt;/diggs:LocationUncertainty&gt;</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -384,6 +923,19 @@
       <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -428,7 +980,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -443,6 +995,12 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -780,15 +1338,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95993B7D-8928-1644-AAE9-9E02DA6FA1A6}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17" thickBottom="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.33203125" style="3" customWidth="1"/>
     <col min="2" max="2" width="36.1640625" style="3" customWidth="1"/>
     <col min="3" max="3" width="48.6640625" style="3" customWidth="1"/>
     <col min="4" max="4" width="45.5" style="3" customWidth="1"/>
-    <col min="5" max="5" width="61.1640625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="59.83203125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="61.83203125" style="7" customWidth="1"/>
+    <col min="6" max="6" width="59.83203125" style="7" customWidth="1"/>
     <col min="7" max="16384" width="10.83203125" style="4"/>
   </cols>
   <sheetData>
@@ -805,7 +1363,7 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -825,14 +1383,14 @@
       <c r="D2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="7" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="138" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="120" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -845,10 +1403,10 @@
       <c r="D3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="7" t="s">
         <v>12</v>
       </c>
     </row>
@@ -865,10 +1423,10 @@
       <c r="D4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="7" t="s">
         <v>19</v>
       </c>
     </row>
@@ -885,14 +1443,14 @@
       <c r="D5" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="7" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="373" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="329" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>45</v>
       </c>
@@ -905,119 +1463,393 @@
       <c r="D6" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="341" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="286" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>57</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>58</v>
+        <v>134</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="7" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="8" spans="1:6" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E8" s="3"/>
-    </row>
-    <row r="9" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="35" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="35" thickBot="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="61" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="69" thickBot="1" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="106" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>34</v>
+        <v>59</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>60</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>36</v>
+        <v>61</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="120" thickBot="1" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="286" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>61</v>
+        <v>65</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>66</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="120" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="91" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="35" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="137" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="91" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="357" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="407" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="136" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="357" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="76" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="409.6" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="121" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="151" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>148</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B12" r:id="rId1" xr:uid="{4B342BBF-B0EB-C941-B8B4-3FA18C9FDB80}"/>
+    <hyperlink ref="B11" r:id="rId1" xr:uid="{4B342BBF-B0EB-C941-B8B4-3FA18C9FDB80}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>